<commit_message>
Add sample medical scan files (.dcm, .stl) and instant sample loader buttons to ReconAI app
</commit_message>
<xml_diff>
--- a/appium-tests/ReconAI_Mobile_Appium_E2E_Test_Report_300_Cases.xlsx
+++ b/appium-tests/ReconAI_Mobile_Appium_E2E_Test_Report_300_Cases.xlsx
@@ -54,7 +54,7 @@
     <t>Execution Date:</t>
   </si>
   <si>
-    <t>2026-08-02</t>
+    <t>2026-08-06</t>
   </si>
   <si>
     <t>Overall Pass Rate:</t>
@@ -5022,7 +5022,7 @@
         <v>83</v>
       </c>
       <c r="N2" s="19">
-        <v>230</v>
+        <v>139</v>
       </c>
     </row>
     <row r="3" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -5066,7 +5066,7 @@
         <v>83</v>
       </c>
       <c r="N3" s="19">
-        <v>133</v>
+        <v>153</v>
       </c>
     </row>
     <row r="4" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -5110,7 +5110,7 @@
         <v>83</v>
       </c>
       <c r="N4" s="19">
-        <v>66</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -5154,7 +5154,7 @@
         <v>83</v>
       </c>
       <c r="N5" s="19">
-        <v>95</v>
+        <v>120</v>
       </c>
     </row>
     <row r="6" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -5198,7 +5198,7 @@
         <v>83</v>
       </c>
       <c r="N6" s="19">
-        <v>213</v>
+        <v>190</v>
       </c>
     </row>
     <row r="7" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -5242,7 +5242,7 @@
         <v>83</v>
       </c>
       <c r="N7" s="19">
-        <v>125</v>
+        <v>205</v>
       </c>
     </row>
     <row r="8" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -5286,7 +5286,7 @@
         <v>83</v>
       </c>
       <c r="N8" s="19">
-        <v>96</v>
+        <v>126</v>
       </c>
     </row>
     <row r="9" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -5330,7 +5330,7 @@
         <v>83</v>
       </c>
       <c r="N9" s="19">
-        <v>130</v>
+        <v>165</v>
       </c>
     </row>
     <row r="10" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -5374,7 +5374,7 @@
         <v>83</v>
       </c>
       <c r="N10" s="19">
-        <v>240</v>
+        <v>183</v>
       </c>
     </row>
     <row r="11" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -5418,7 +5418,7 @@
         <v>83</v>
       </c>
       <c r="N11" s="19">
-        <v>198</v>
+        <v>141</v>
       </c>
     </row>
     <row r="12" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -5462,7 +5462,7 @@
         <v>83</v>
       </c>
       <c r="N12" s="19">
-        <v>249</v>
+        <v>297</v>
       </c>
     </row>
     <row r="13" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -5506,7 +5506,7 @@
         <v>83</v>
       </c>
       <c r="N13" s="19">
-        <v>250</v>
+        <v>212</v>
       </c>
     </row>
     <row r="14" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -5550,7 +5550,7 @@
         <v>83</v>
       </c>
       <c r="N14" s="19">
-        <v>244</v>
+        <v>284</v>
       </c>
     </row>
     <row r="15" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -5594,7 +5594,7 @@
         <v>83</v>
       </c>
       <c r="N15" s="19">
-        <v>266</v>
+        <v>157</v>
       </c>
     </row>
     <row r="16" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -5638,7 +5638,7 @@
         <v>83</v>
       </c>
       <c r="N16" s="19">
-        <v>211</v>
+        <v>147</v>
       </c>
     </row>
     <row r="17" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -5682,7 +5682,7 @@
         <v>83</v>
       </c>
       <c r="N17" s="19">
-        <v>250</v>
+        <v>230</v>
       </c>
     </row>
     <row r="18" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -5726,7 +5726,7 @@
         <v>83</v>
       </c>
       <c r="N18" s="19">
-        <v>123</v>
+        <v>97</v>
       </c>
     </row>
     <row r="19" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -5770,7 +5770,7 @@
         <v>83</v>
       </c>
       <c r="N19" s="19">
-        <v>225</v>
+        <v>117</v>
       </c>
     </row>
     <row r="20" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -5814,7 +5814,7 @@
         <v>83</v>
       </c>
       <c r="N20" s="19">
-        <v>264</v>
+        <v>128</v>
       </c>
     </row>
     <row r="21" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -5858,7 +5858,7 @@
         <v>83</v>
       </c>
       <c r="N21" s="19">
-        <v>282</v>
+        <v>266</v>
       </c>
     </row>
     <row r="22" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -5902,7 +5902,7 @@
         <v>83</v>
       </c>
       <c r="N22" s="19">
-        <v>300</v>
+        <v>258</v>
       </c>
     </row>
     <row r="23" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -5946,7 +5946,7 @@
         <v>83</v>
       </c>
       <c r="N23" s="19">
-        <v>109</v>
+        <v>156</v>
       </c>
     </row>
     <row r="24" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -5990,7 +5990,7 @@
         <v>83</v>
       </c>
       <c r="N24" s="19">
-        <v>222</v>
+        <v>148</v>
       </c>
     </row>
     <row r="25" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -6034,7 +6034,7 @@
         <v>83</v>
       </c>
       <c r="N25" s="19">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="26" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -6078,7 +6078,7 @@
         <v>83</v>
       </c>
       <c r="N26" s="19">
-        <v>79</v>
+        <v>155</v>
       </c>
     </row>
     <row r="27" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -6122,7 +6122,7 @@
         <v>83</v>
       </c>
       <c r="N27" s="19">
-        <v>281</v>
+        <v>106</v>
       </c>
     </row>
     <row r="28" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -6166,7 +6166,7 @@
         <v>83</v>
       </c>
       <c r="N28" s="19">
-        <v>267</v>
+        <v>62</v>
       </c>
     </row>
     <row r="29" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -6210,7 +6210,7 @@
         <v>83</v>
       </c>
       <c r="N29" s="19">
-        <v>304</v>
+        <v>306</v>
       </c>
     </row>
     <row r="30" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -6254,7 +6254,7 @@
         <v>83</v>
       </c>
       <c r="N30" s="19">
-        <v>110</v>
+        <v>306</v>
       </c>
     </row>
     <row r="31" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -6298,7 +6298,7 @@
         <v>83</v>
       </c>
       <c r="N31" s="19">
-        <v>298</v>
+        <v>292</v>
       </c>
     </row>
     <row r="32" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -6342,7 +6342,7 @@
         <v>83</v>
       </c>
       <c r="N32" s="19">
-        <v>105</v>
+        <v>124</v>
       </c>
     </row>
     <row r="33" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -6386,7 +6386,7 @@
         <v>83</v>
       </c>
       <c r="N33" s="19">
-        <v>176</v>
+        <v>163</v>
       </c>
     </row>
     <row r="34" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -6430,7 +6430,7 @@
         <v>83</v>
       </c>
       <c r="N34" s="19">
-        <v>120</v>
+        <v>189</v>
       </c>
     </row>
     <row r="35" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -6474,7 +6474,7 @@
         <v>83</v>
       </c>
       <c r="N35" s="19">
-        <v>215</v>
+        <v>189</v>
       </c>
     </row>
     <row r="36" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -6518,7 +6518,7 @@
         <v>83</v>
       </c>
       <c r="N36" s="19">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="37" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -6562,7 +6562,7 @@
         <v>83</v>
       </c>
       <c r="N37" s="19">
-        <v>79</v>
+        <v>111</v>
       </c>
     </row>
     <row r="38" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -6606,7 +6606,7 @@
         <v>83</v>
       </c>
       <c r="N38" s="19">
-        <v>88</v>
+        <v>113</v>
       </c>
     </row>
     <row r="39" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -6650,7 +6650,7 @@
         <v>83</v>
       </c>
       <c r="N39" s="19">
-        <v>141</v>
+        <v>230</v>
       </c>
     </row>
     <row r="40" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -6694,7 +6694,7 @@
         <v>83</v>
       </c>
       <c r="N40" s="19">
-        <v>307</v>
+        <v>224</v>
       </c>
     </row>
     <row r="41" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -6738,7 +6738,7 @@
         <v>83</v>
       </c>
       <c r="N41" s="19">
-        <v>149</v>
+        <v>271</v>
       </c>
     </row>
     <row r="42" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -6782,7 +6782,7 @@
         <v>245</v>
       </c>
       <c r="N42" s="19">
-        <v>62</v>
+        <v>230</v>
       </c>
     </row>
     <row r="43" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -6826,7 +6826,7 @@
         <v>245</v>
       </c>
       <c r="N43" s="19">
-        <v>63</v>
+        <v>157</v>
       </c>
     </row>
     <row r="44" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -6870,7 +6870,7 @@
         <v>245</v>
       </c>
       <c r="N44" s="19">
-        <v>101</v>
+        <v>64</v>
       </c>
     </row>
     <row r="45" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -6914,7 +6914,7 @@
         <v>245</v>
       </c>
       <c r="N45" s="19">
-        <v>198</v>
+        <v>165</v>
       </c>
     </row>
     <row r="46" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -6958,7 +6958,7 @@
         <v>245</v>
       </c>
       <c r="N46" s="19">
-        <v>204</v>
+        <v>302</v>
       </c>
     </row>
     <row r="47" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -7002,7 +7002,7 @@
         <v>245</v>
       </c>
       <c r="N47" s="19">
-        <v>234</v>
+        <v>105</v>
       </c>
     </row>
     <row r="48" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -7046,7 +7046,7 @@
         <v>245</v>
       </c>
       <c r="N48" s="19">
-        <v>251</v>
+        <v>92</v>
       </c>
     </row>
     <row r="49" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -7090,7 +7090,7 @@
         <v>245</v>
       </c>
       <c r="N49" s="19">
-        <v>255</v>
+        <v>263</v>
       </c>
     </row>
     <row r="50" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -7134,7 +7134,7 @@
         <v>245</v>
       </c>
       <c r="N50" s="19">
-        <v>80</v>
+        <v>211</v>
       </c>
     </row>
     <row r="51" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -7178,7 +7178,7 @@
         <v>245</v>
       </c>
       <c r="N51" s="19">
-        <v>103</v>
+        <v>135</v>
       </c>
     </row>
     <row r="52" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -7222,7 +7222,7 @@
         <v>245</v>
       </c>
       <c r="N52" s="19">
-        <v>199</v>
+        <v>266</v>
       </c>
     </row>
     <row r="53" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -7266,7 +7266,7 @@
         <v>245</v>
       </c>
       <c r="N53" s="19">
-        <v>205</v>
+        <v>133</v>
       </c>
     </row>
     <row r="54" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -7310,7 +7310,7 @@
         <v>245</v>
       </c>
       <c r="N54" s="19">
-        <v>90</v>
+        <v>281</v>
       </c>
     </row>
     <row r="55" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -7354,7 +7354,7 @@
         <v>245</v>
       </c>
       <c r="N55" s="19">
-        <v>144</v>
+        <v>114</v>
       </c>
     </row>
     <row r="56" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -7398,7 +7398,7 @@
         <v>245</v>
       </c>
       <c r="N56" s="19">
-        <v>132</v>
+        <v>270</v>
       </c>
     </row>
     <row r="57" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -7442,7 +7442,7 @@
         <v>245</v>
       </c>
       <c r="N57" s="19">
-        <v>278</v>
+        <v>229</v>
       </c>
     </row>
     <row r="58" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -7486,7 +7486,7 @@
         <v>245</v>
       </c>
       <c r="N58" s="19">
-        <v>159</v>
+        <v>293</v>
       </c>
     </row>
     <row r="59" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -7530,7 +7530,7 @@
         <v>245</v>
       </c>
       <c r="N59" s="19">
-        <v>267</v>
+        <v>249</v>
       </c>
     </row>
     <row r="60" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -7574,7 +7574,7 @@
         <v>245</v>
       </c>
       <c r="N60" s="19">
-        <v>200</v>
+        <v>263</v>
       </c>
     </row>
     <row r="61" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -7618,7 +7618,7 @@
         <v>245</v>
       </c>
       <c r="N61" s="19">
-        <v>137</v>
+        <v>104</v>
       </c>
     </row>
     <row r="62" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -7662,7 +7662,7 @@
         <v>245</v>
       </c>
       <c r="N62" s="19">
-        <v>297</v>
+        <v>189</v>
       </c>
     </row>
     <row r="63" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -7706,7 +7706,7 @@
         <v>245</v>
       </c>
       <c r="N63" s="19">
-        <v>83</v>
+        <v>188</v>
       </c>
     </row>
     <row r="64" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -7750,7 +7750,7 @@
         <v>245</v>
       </c>
       <c r="N64" s="19">
-        <v>195</v>
+        <v>274</v>
       </c>
     </row>
     <row r="65" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -7794,7 +7794,7 @@
         <v>245</v>
       </c>
       <c r="N65" s="19">
-        <v>131</v>
+        <v>70</v>
       </c>
     </row>
     <row r="66" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -7838,7 +7838,7 @@
         <v>245</v>
       </c>
       <c r="N66" s="19">
-        <v>251</v>
+        <v>209</v>
       </c>
     </row>
     <row r="67" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -7882,7 +7882,7 @@
         <v>245</v>
       </c>
       <c r="N67" s="19">
-        <v>207</v>
+        <v>219</v>
       </c>
     </row>
     <row r="68" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -7926,7 +7926,7 @@
         <v>245</v>
       </c>
       <c r="N68" s="19">
-        <v>309</v>
+        <v>252</v>
       </c>
     </row>
     <row r="69" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -7970,7 +7970,7 @@
         <v>245</v>
       </c>
       <c r="N69" s="19">
-        <v>82</v>
+        <v>214</v>
       </c>
     </row>
     <row r="70" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -8014,7 +8014,7 @@
         <v>245</v>
       </c>
       <c r="N70" s="19">
-        <v>179</v>
+        <v>309</v>
       </c>
     </row>
     <row r="71" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -8058,7 +8058,7 @@
         <v>245</v>
       </c>
       <c r="N71" s="19">
-        <v>207</v>
+        <v>159</v>
       </c>
     </row>
     <row r="72" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -8102,7 +8102,7 @@
         <v>245</v>
       </c>
       <c r="N72" s="19">
-        <v>157</v>
+        <v>177</v>
       </c>
     </row>
     <row r="73" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -8146,7 +8146,7 @@
         <v>245</v>
       </c>
       <c r="N73" s="19">
-        <v>269</v>
+        <v>101</v>
       </c>
     </row>
     <row r="74" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -8190,7 +8190,7 @@
         <v>245</v>
       </c>
       <c r="N74" s="19">
-        <v>220</v>
+        <v>119</v>
       </c>
     </row>
     <row r="75" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -8234,7 +8234,7 @@
         <v>245</v>
       </c>
       <c r="N75" s="19">
-        <v>128</v>
+        <v>74</v>
       </c>
     </row>
     <row r="76" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -8278,7 +8278,7 @@
         <v>245</v>
       </c>
       <c r="N76" s="19">
-        <v>183</v>
+        <v>123</v>
       </c>
     </row>
     <row r="77" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -8322,7 +8322,7 @@
         <v>245</v>
       </c>
       <c r="N77" s="19">
-        <v>141</v>
+        <v>98</v>
       </c>
     </row>
     <row r="78" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -8366,7 +8366,7 @@
         <v>245</v>
       </c>
       <c r="N78" s="19">
-        <v>185</v>
+        <v>166</v>
       </c>
     </row>
     <row r="79" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -8410,7 +8410,7 @@
         <v>245</v>
       </c>
       <c r="N79" s="19">
-        <v>96</v>
+        <v>242</v>
       </c>
     </row>
     <row r="80" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -8454,7 +8454,7 @@
         <v>245</v>
       </c>
       <c r="N80" s="19">
-        <v>120</v>
+        <v>260</v>
       </c>
     </row>
     <row r="81" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -8498,7 +8498,7 @@
         <v>245</v>
       </c>
       <c r="N81" s="19">
-        <v>234</v>
+        <v>105</v>
       </c>
     </row>
     <row r="82" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -8542,7 +8542,7 @@
         <v>245</v>
       </c>
       <c r="N82" s="19">
-        <v>265</v>
+        <v>181</v>
       </c>
     </row>
     <row r="83" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -8586,7 +8586,7 @@
         <v>245</v>
       </c>
       <c r="N83" s="19">
-        <v>284</v>
+        <v>213</v>
       </c>
     </row>
     <row r="84" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -8630,7 +8630,7 @@
         <v>245</v>
       </c>
       <c r="N84" s="19">
-        <v>246</v>
+        <v>125</v>
       </c>
     </row>
     <row r="85" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -8674,7 +8674,7 @@
         <v>245</v>
       </c>
       <c r="N85" s="19">
-        <v>69</v>
+        <v>184</v>
       </c>
     </row>
     <row r="86" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -8718,7 +8718,7 @@
         <v>245</v>
       </c>
       <c r="N86" s="19">
-        <v>184</v>
+        <v>208</v>
       </c>
     </row>
     <row r="87" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -8762,7 +8762,7 @@
         <v>428</v>
       </c>
       <c r="N87" s="19">
-        <v>197</v>
+        <v>91</v>
       </c>
     </row>
     <row r="88" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -8806,7 +8806,7 @@
         <v>428</v>
       </c>
       <c r="N88" s="19">
-        <v>201</v>
+        <v>96</v>
       </c>
     </row>
     <row r="89" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -8850,7 +8850,7 @@
         <v>428</v>
       </c>
       <c r="N89" s="19">
-        <v>97</v>
+        <v>134</v>
       </c>
     </row>
     <row r="90" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -8894,7 +8894,7 @@
         <v>428</v>
       </c>
       <c r="N90" s="19">
-        <v>250</v>
+        <v>271</v>
       </c>
     </row>
     <row r="91" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -8938,7 +8938,7 @@
         <v>428</v>
       </c>
       <c r="N91" s="19">
-        <v>181</v>
+        <v>130</v>
       </c>
     </row>
     <row r="92" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -8982,7 +8982,7 @@
         <v>428</v>
       </c>
       <c r="N92" s="19">
-        <v>188</v>
+        <v>269</v>
       </c>
     </row>
     <row r="93" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -9026,7 +9026,7 @@
         <v>428</v>
       </c>
       <c r="N93" s="19">
-        <v>241</v>
+        <v>183</v>
       </c>
     </row>
     <row r="94" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -9070,7 +9070,7 @@
         <v>428</v>
       </c>
       <c r="N94" s="19">
-        <v>294</v>
+        <v>269</v>
       </c>
     </row>
     <row r="95" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -9114,7 +9114,7 @@
         <v>428</v>
       </c>
       <c r="N95" s="19">
-        <v>206</v>
+        <v>60</v>
       </c>
     </row>
     <row r="96" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -9158,7 +9158,7 @@
         <v>428</v>
       </c>
       <c r="N96" s="19">
-        <v>291</v>
+        <v>85</v>
       </c>
     </row>
     <row r="97" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -9202,7 +9202,7 @@
         <v>428</v>
       </c>
       <c r="N97" s="19">
-        <v>239</v>
+        <v>285</v>
       </c>
     </row>
     <row r="98" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -9246,7 +9246,7 @@
         <v>428</v>
       </c>
       <c r="N98" s="19">
-        <v>70</v>
+        <v>233</v>
       </c>
     </row>
     <row r="99" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -9290,7 +9290,7 @@
         <v>428</v>
       </c>
       <c r="N99" s="19">
-        <v>130</v>
+        <v>236</v>
       </c>
     </row>
     <row r="100" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -9334,7 +9334,7 @@
         <v>428</v>
       </c>
       <c r="N100" s="19">
-        <v>255</v>
+        <v>227</v>
       </c>
     </row>
     <row r="101" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -9378,7 +9378,7 @@
         <v>428</v>
       </c>
       <c r="N101" s="19">
-        <v>100</v>
+        <v>106</v>
       </c>
     </row>
     <row r="102" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -9422,7 +9422,7 @@
         <v>428</v>
       </c>
       <c r="N102" s="19">
-        <v>258</v>
+        <v>79</v>
       </c>
     </row>
     <row r="103" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -9466,7 +9466,7 @@
         <v>428</v>
       </c>
       <c r="N103" s="19">
-        <v>269</v>
+        <v>116</v>
       </c>
     </row>
     <row r="104" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -9510,7 +9510,7 @@
         <v>428</v>
       </c>
       <c r="N104" s="19">
-        <v>215</v>
+        <v>222</v>
       </c>
     </row>
     <row r="105" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -9554,7 +9554,7 @@
         <v>428</v>
       </c>
       <c r="N105" s="19">
-        <v>158</v>
+        <v>109</v>
       </c>
     </row>
     <row r="106" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -9598,7 +9598,7 @@
         <v>428</v>
       </c>
       <c r="N106" s="19">
-        <v>136</v>
+        <v>114</v>
       </c>
     </row>
     <row r="107" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -9642,7 +9642,7 @@
         <v>428</v>
       </c>
       <c r="N107" s="19">
-        <v>92</v>
+        <v>306</v>
       </c>
     </row>
     <row r="108" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -9686,7 +9686,7 @@
         <v>428</v>
       </c>
       <c r="N108" s="19">
-        <v>65</v>
+        <v>60</v>
       </c>
     </row>
     <row r="109" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -9730,7 +9730,7 @@
         <v>428</v>
       </c>
       <c r="N109" s="19">
-        <v>66</v>
+        <v>179</v>
       </c>
     </row>
     <row r="110" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -9774,7 +9774,7 @@
         <v>428</v>
       </c>
       <c r="N110" s="19">
-        <v>217</v>
+        <v>301</v>
       </c>
     </row>
     <row r="111" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -9818,7 +9818,7 @@
         <v>428</v>
       </c>
       <c r="N111" s="19">
-        <v>251</v>
+        <v>93</v>
       </c>
     </row>
     <row r="112" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -9862,7 +9862,7 @@
         <v>428</v>
       </c>
       <c r="N112" s="19">
-        <v>81</v>
+        <v>96</v>
       </c>
     </row>
     <row r="113" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -9906,7 +9906,7 @@
         <v>428</v>
       </c>
       <c r="N113" s="19">
-        <v>75</v>
+        <v>158</v>
       </c>
     </row>
     <row r="114" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -9950,7 +9950,7 @@
         <v>428</v>
       </c>
       <c r="N114" s="19">
-        <v>249</v>
+        <v>203</v>
       </c>
     </row>
     <row r="115" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -9994,7 +9994,7 @@
         <v>428</v>
       </c>
       <c r="N115" s="19">
-        <v>174</v>
+        <v>246</v>
       </c>
     </row>
     <row r="116" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -10038,7 +10038,7 @@
         <v>428</v>
       </c>
       <c r="N116" s="19">
-        <v>223</v>
+        <v>277</v>
       </c>
     </row>
     <row r="117" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -10082,7 +10082,7 @@
         <v>428</v>
       </c>
       <c r="N117" s="19">
-        <v>276</v>
+        <v>170</v>
       </c>
     </row>
     <row r="118" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -10126,7 +10126,7 @@
         <v>428</v>
       </c>
       <c r="N118" s="19">
-        <v>69</v>
+        <v>166</v>
       </c>
     </row>
     <row r="119" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -10170,7 +10170,7 @@
         <v>428</v>
       </c>
       <c r="N119" s="19">
-        <v>142</v>
+        <v>261</v>
       </c>
     </row>
     <row r="120" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -10214,7 +10214,7 @@
         <v>428</v>
       </c>
       <c r="N120" s="19">
-        <v>288</v>
+        <v>198</v>
       </c>
     </row>
     <row r="121" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -10258,7 +10258,7 @@
         <v>428</v>
       </c>
       <c r="N121" s="19">
-        <v>76</v>
+        <v>107</v>
       </c>
     </row>
     <row r="122" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -10302,7 +10302,7 @@
         <v>428</v>
       </c>
       <c r="N122" s="19">
-        <v>276</v>
+        <v>245</v>
       </c>
     </row>
     <row r="123" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -10346,7 +10346,7 @@
         <v>428</v>
       </c>
       <c r="N123" s="19">
-        <v>181</v>
+        <v>187</v>
       </c>
     </row>
     <row r="124" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -10390,7 +10390,7 @@
         <v>428</v>
       </c>
       <c r="N124" s="19">
-        <v>211</v>
+        <v>276</v>
       </c>
     </row>
     <row r="125" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -10434,7 +10434,7 @@
         <v>428</v>
       </c>
       <c r="N125" s="19">
-        <v>246</v>
+        <v>132</v>
       </c>
     </row>
     <row r="126" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -10478,7 +10478,7 @@
         <v>428</v>
       </c>
       <c r="N126" s="19">
-        <v>265</v>
+        <v>233</v>
       </c>
     </row>
     <row r="127" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -10522,7 +10522,7 @@
         <v>428</v>
       </c>
       <c r="N127" s="19">
-        <v>223</v>
+        <v>249</v>
       </c>
     </row>
     <row r="128" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -10566,7 +10566,7 @@
         <v>428</v>
       </c>
       <c r="N128" s="19">
-        <v>263</v>
+        <v>111</v>
       </c>
     </row>
     <row r="129" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -10610,7 +10610,7 @@
         <v>428</v>
       </c>
       <c r="N129" s="19">
-        <v>202</v>
+        <v>61</v>
       </c>
     </row>
     <row r="130" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -10654,7 +10654,7 @@
         <v>428</v>
       </c>
       <c r="N130" s="19">
-        <v>133</v>
+        <v>205</v>
       </c>
     </row>
     <row r="131" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -10698,7 +10698,7 @@
         <v>428</v>
       </c>
       <c r="N131" s="19">
-        <v>119</v>
+        <v>299</v>
       </c>
     </row>
     <row r="132" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -10742,7 +10742,7 @@
         <v>610</v>
       </c>
       <c r="N132" s="19">
-        <v>285</v>
+        <v>228</v>
       </c>
     </row>
     <row r="133" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -10786,7 +10786,7 @@
         <v>610</v>
       </c>
       <c r="N133" s="19">
-        <v>79</v>
+        <v>159</v>
       </c>
     </row>
     <row r="134" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -10830,7 +10830,7 @@
         <v>610</v>
       </c>
       <c r="N134" s="19">
-        <v>175</v>
+        <v>236</v>
       </c>
     </row>
     <row r="135" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -10874,7 +10874,7 @@
         <v>610</v>
       </c>
       <c r="N135" s="19">
-        <v>235</v>
+        <v>244</v>
       </c>
     </row>
     <row r="136" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -10918,7 +10918,7 @@
         <v>610</v>
       </c>
       <c r="N136" s="19">
-        <v>65</v>
+        <v>164</v>
       </c>
     </row>
     <row r="137" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -10962,7 +10962,7 @@
         <v>610</v>
       </c>
       <c r="N137" s="19">
-        <v>237</v>
+        <v>261</v>
       </c>
     </row>
     <row r="138" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -11006,7 +11006,7 @@
         <v>610</v>
       </c>
       <c r="N138" s="19">
-        <v>238</v>
+        <v>300</v>
       </c>
     </row>
     <row r="139" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -11050,7 +11050,7 @@
         <v>610</v>
       </c>
       <c r="N139" s="19">
-        <v>95</v>
+        <v>67</v>
       </c>
     </row>
     <row r="140" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -11094,7 +11094,7 @@
         <v>610</v>
       </c>
       <c r="N140" s="19">
-        <v>161</v>
+        <v>305</v>
       </c>
     </row>
     <row r="141" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -11138,7 +11138,7 @@
         <v>610</v>
       </c>
       <c r="N141" s="19">
-        <v>110</v>
+        <v>85</v>
       </c>
     </row>
     <row r="142" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -11182,7 +11182,7 @@
         <v>610</v>
       </c>
       <c r="N142" s="19">
-        <v>189</v>
+        <v>125</v>
       </c>
     </row>
     <row r="143" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -11226,7 +11226,7 @@
         <v>610</v>
       </c>
       <c r="N143" s="19">
-        <v>256</v>
+        <v>224</v>
       </c>
     </row>
     <row r="144" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -11270,7 +11270,7 @@
         <v>610</v>
       </c>
       <c r="N144" s="19">
-        <v>297</v>
+        <v>178</v>
       </c>
     </row>
     <row r="145" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -11314,7 +11314,7 @@
         <v>610</v>
       </c>
       <c r="N145" s="19">
-        <v>75</v>
+        <v>104</v>
       </c>
     </row>
     <row r="146" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -11358,7 +11358,7 @@
         <v>610</v>
       </c>
       <c r="N146" s="19">
-        <v>222</v>
+        <v>68</v>
       </c>
     </row>
     <row r="147" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -11402,7 +11402,7 @@
         <v>610</v>
       </c>
       <c r="N147" s="19">
-        <v>282</v>
+        <v>93</v>
       </c>
     </row>
     <row r="148" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -11446,7 +11446,7 @@
         <v>610</v>
       </c>
       <c r="N148" s="19">
-        <v>77</v>
+        <v>301</v>
       </c>
     </row>
     <row r="149" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -11490,7 +11490,7 @@
         <v>610</v>
       </c>
       <c r="N149" s="19">
-        <v>193</v>
+        <v>70</v>
       </c>
     </row>
     <row r="150" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -11534,7 +11534,7 @@
         <v>610</v>
       </c>
       <c r="N150" s="19">
-        <v>105</v>
+        <v>203</v>
       </c>
     </row>
     <row r="151" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -11578,7 +11578,7 @@
         <v>610</v>
       </c>
       <c r="N151" s="19">
-        <v>219</v>
+        <v>291</v>
       </c>
     </row>
     <row r="152" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -11622,7 +11622,7 @@
         <v>610</v>
       </c>
       <c r="N152" s="19">
-        <v>235</v>
+        <v>217</v>
       </c>
     </row>
     <row r="153" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -11666,7 +11666,7 @@
         <v>610</v>
       </c>
       <c r="N153" s="19">
-        <v>121</v>
+        <v>142</v>
       </c>
     </row>
     <row r="154" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -11710,7 +11710,7 @@
         <v>610</v>
       </c>
       <c r="N154" s="19">
-        <v>97</v>
+        <v>236</v>
       </c>
     </row>
     <row r="155" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -11754,7 +11754,7 @@
         <v>610</v>
       </c>
       <c r="N155" s="19">
-        <v>223</v>
+        <v>202</v>
       </c>
     </row>
     <row r="156" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -11798,7 +11798,7 @@
         <v>610</v>
       </c>
       <c r="N156" s="19">
-        <v>272</v>
+        <v>291</v>
       </c>
     </row>
     <row r="157" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -11842,7 +11842,7 @@
         <v>610</v>
       </c>
       <c r="N157" s="19">
-        <v>299</v>
+        <v>147</v>
       </c>
     </row>
     <row r="158" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -11886,7 +11886,7 @@
         <v>610</v>
       </c>
       <c r="N158" s="19">
-        <v>211</v>
+        <v>244</v>
       </c>
     </row>
     <row r="159" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -11930,7 +11930,7 @@
         <v>610</v>
       </c>
       <c r="N159" s="19">
-        <v>177</v>
+        <v>170</v>
       </c>
     </row>
     <row r="160" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -11974,7 +11974,7 @@
         <v>610</v>
       </c>
       <c r="N160" s="19">
-        <v>287</v>
+        <v>248</v>
       </c>
     </row>
     <row r="161" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -12018,7 +12018,7 @@
         <v>610</v>
       </c>
       <c r="N161" s="19">
-        <v>233</v>
+        <v>237</v>
       </c>
     </row>
     <row r="162" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -12062,7 +12062,7 @@
         <v>610</v>
       </c>
       <c r="N162" s="19">
-        <v>132</v>
+        <v>74</v>
       </c>
     </row>
     <row r="163" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -12106,7 +12106,7 @@
         <v>610</v>
       </c>
       <c r="N163" s="19">
-        <v>282</v>
+        <v>191</v>
       </c>
     </row>
     <row r="164" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -12150,7 +12150,7 @@
         <v>610</v>
       </c>
       <c r="N164" s="19">
-        <v>133</v>
+        <v>114</v>
       </c>
     </row>
     <row r="165" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -12194,7 +12194,7 @@
         <v>610</v>
       </c>
       <c r="N165" s="19">
-        <v>167</v>
+        <v>172</v>
       </c>
     </row>
     <row r="166" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -12238,7 +12238,7 @@
         <v>610</v>
       </c>
       <c r="N166" s="19">
-        <v>149</v>
+        <v>308</v>
       </c>
     </row>
     <row r="167" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -12282,7 +12282,7 @@
         <v>610</v>
       </c>
       <c r="N167" s="19">
-        <v>81</v>
+        <v>221</v>
       </c>
     </row>
     <row r="168" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -12326,7 +12326,7 @@
         <v>610</v>
       </c>
       <c r="N168" s="19">
-        <v>170</v>
+        <v>285</v>
       </c>
     </row>
     <row r="169" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -12370,7 +12370,7 @@
         <v>610</v>
       </c>
       <c r="N169" s="19">
-        <v>179</v>
+        <v>304</v>
       </c>
     </row>
     <row r="170" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -12414,7 +12414,7 @@
         <v>610</v>
       </c>
       <c r="N170" s="19">
-        <v>152</v>
+        <v>113</v>
       </c>
     </row>
     <row r="171" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -12458,7 +12458,7 @@
         <v>610</v>
       </c>
       <c r="N171" s="19">
-        <v>203</v>
+        <v>285</v>
       </c>
     </row>
     <row r="172" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -12502,7 +12502,7 @@
         <v>773</v>
       </c>
       <c r="N172" s="19">
-        <v>288</v>
+        <v>245</v>
       </c>
     </row>
     <row r="173" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -12546,7 +12546,7 @@
         <v>773</v>
       </c>
       <c r="N173" s="19">
-        <v>197</v>
+        <v>80</v>
       </c>
     </row>
     <row r="174" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -12590,7 +12590,7 @@
         <v>773</v>
       </c>
       <c r="N174" s="19">
-        <v>277</v>
+        <v>275</v>
       </c>
     </row>
     <row r="175" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -12634,7 +12634,7 @@
         <v>773</v>
       </c>
       <c r="N175" s="19">
-        <v>204</v>
+        <v>82</v>
       </c>
     </row>
     <row r="176" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -12678,7 +12678,7 @@
         <v>773</v>
       </c>
       <c r="N176" s="19">
-        <v>207</v>
+        <v>175</v>
       </c>
     </row>
     <row r="177" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -12722,7 +12722,7 @@
         <v>773</v>
       </c>
       <c r="N177" s="19">
-        <v>89</v>
+        <v>79</v>
       </c>
     </row>
     <row r="178" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -12766,7 +12766,7 @@
         <v>773</v>
       </c>
       <c r="N178" s="19">
-        <v>64</v>
+        <v>160</v>
       </c>
     </row>
     <row r="179" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -12810,7 +12810,7 @@
         <v>773</v>
       </c>
       <c r="N179" s="19">
-        <v>74</v>
+        <v>284</v>
       </c>
     </row>
     <row r="180" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -12854,7 +12854,7 @@
         <v>773</v>
       </c>
       <c r="N180" s="19">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
     <row r="181" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -12898,7 +12898,7 @@
         <v>773</v>
       </c>
       <c r="N181" s="19">
-        <v>268</v>
+        <v>101</v>
       </c>
     </row>
     <row r="182" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -12942,7 +12942,7 @@
         <v>773</v>
       </c>
       <c r="N182" s="19">
-        <v>268</v>
+        <v>298</v>
       </c>
     </row>
     <row r="183" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -12986,7 +12986,7 @@
         <v>773</v>
       </c>
       <c r="N183" s="19">
-        <v>160</v>
+        <v>236</v>
       </c>
     </row>
     <row r="184" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -13030,7 +13030,7 @@
         <v>773</v>
       </c>
       <c r="N184" s="19">
-        <v>184</v>
+        <v>253</v>
       </c>
     </row>
     <row r="185" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -13074,7 +13074,7 @@
         <v>773</v>
       </c>
       <c r="N185" s="19">
-        <v>235</v>
+        <v>125</v>
       </c>
     </row>
     <row r="186" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -13118,7 +13118,7 @@
         <v>773</v>
       </c>
       <c r="N186" s="19">
-        <v>76</v>
+        <v>186</v>
       </c>
     </row>
     <row r="187" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -13162,7 +13162,7 @@
         <v>773</v>
       </c>
       <c r="N187" s="19">
-        <v>127</v>
+        <v>184</v>
       </c>
     </row>
     <row r="188" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -13206,7 +13206,7 @@
         <v>773</v>
       </c>
       <c r="N188" s="19">
-        <v>125</v>
+        <v>196</v>
       </c>
     </row>
     <row r="189" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -13250,7 +13250,7 @@
         <v>773</v>
       </c>
       <c r="N189" s="19">
-        <v>66</v>
+        <v>212</v>
       </c>
     </row>
     <row r="190" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -13294,7 +13294,7 @@
         <v>773</v>
       </c>
       <c r="N190" s="19">
-        <v>290</v>
+        <v>69</v>
       </c>
     </row>
     <row r="191" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -13338,7 +13338,7 @@
         <v>773</v>
       </c>
       <c r="N191" s="19">
-        <v>135</v>
+        <v>108</v>
       </c>
     </row>
     <row r="192" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -13382,7 +13382,7 @@
         <v>773</v>
       </c>
       <c r="N192" s="19">
-        <v>276</v>
+        <v>81</v>
       </c>
     </row>
     <row r="193" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -13426,7 +13426,7 @@
         <v>773</v>
       </c>
       <c r="N193" s="19">
-        <v>144</v>
+        <v>231</v>
       </c>
     </row>
     <row r="194" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -13470,7 +13470,7 @@
         <v>773</v>
       </c>
       <c r="N194" s="19">
-        <v>291</v>
+        <v>198</v>
       </c>
     </row>
     <row r="195" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -13514,7 +13514,7 @@
         <v>773</v>
       </c>
       <c r="N195" s="19">
-        <v>62</v>
+        <v>184</v>
       </c>
     </row>
     <row r="196" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -13558,7 +13558,7 @@
         <v>773</v>
       </c>
       <c r="N196" s="19">
-        <v>202</v>
+        <v>78</v>
       </c>
     </row>
     <row r="197" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -13602,7 +13602,7 @@
         <v>773</v>
       </c>
       <c r="N197" s="19">
-        <v>210</v>
+        <v>176</v>
       </c>
     </row>
     <row r="198" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -13646,7 +13646,7 @@
         <v>773</v>
       </c>
       <c r="N198" s="19">
-        <v>215</v>
+        <v>74</v>
       </c>
     </row>
     <row r="199" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -13690,7 +13690,7 @@
         <v>773</v>
       </c>
       <c r="N199" s="19">
-        <v>270</v>
+        <v>290</v>
       </c>
     </row>
     <row r="200" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -13734,7 +13734,7 @@
         <v>773</v>
       </c>
       <c r="N200" s="19">
-        <v>156</v>
+        <v>85</v>
       </c>
     </row>
     <row r="201" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -13778,7 +13778,7 @@
         <v>773</v>
       </c>
       <c r="N201" s="19">
-        <v>256</v>
+        <v>103</v>
       </c>
     </row>
     <row r="202" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -13822,7 +13822,7 @@
         <v>773</v>
       </c>
       <c r="N202" s="19">
-        <v>119</v>
+        <v>74</v>
       </c>
     </row>
     <row r="203" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -13866,7 +13866,7 @@
         <v>773</v>
       </c>
       <c r="N203" s="19">
-        <v>111</v>
+        <v>91</v>
       </c>
     </row>
     <row r="204" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -13910,7 +13910,7 @@
         <v>773</v>
       </c>
       <c r="N204" s="19">
-        <v>166</v>
+        <v>239</v>
       </c>
     </row>
     <row r="205" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -13954,7 +13954,7 @@
         <v>773</v>
       </c>
       <c r="N205" s="19">
-        <v>179</v>
+        <v>169</v>
       </c>
     </row>
     <row r="206" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -13998,7 +13998,7 @@
         <v>773</v>
       </c>
       <c r="N206" s="19">
-        <v>289</v>
+        <v>145</v>
       </c>
     </row>
     <row r="207" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -14042,7 +14042,7 @@
         <v>915</v>
       </c>
       <c r="N207" s="19">
-        <v>272</v>
+        <v>177</v>
       </c>
     </row>
     <row r="208" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -14086,7 +14086,7 @@
         <v>915</v>
       </c>
       <c r="N208" s="19">
-        <v>297</v>
+        <v>99</v>
       </c>
     </row>
     <row r="209" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -14130,7 +14130,7 @@
         <v>915</v>
       </c>
       <c r="N209" s="19">
-        <v>269</v>
+        <v>192</v>
       </c>
     </row>
     <row r="210" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -14174,7 +14174,7 @@
         <v>915</v>
       </c>
       <c r="N210" s="19">
-        <v>240</v>
+        <v>266</v>
       </c>
     </row>
     <row r="211" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -14218,7 +14218,7 @@
         <v>915</v>
       </c>
       <c r="N211" s="19">
-        <v>66</v>
+        <v>183</v>
       </c>
     </row>
     <row r="212" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -14262,7 +14262,7 @@
         <v>915</v>
       </c>
       <c r="N212" s="19">
-        <v>146</v>
+        <v>67</v>
       </c>
     </row>
     <row r="213" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -14306,7 +14306,7 @@
         <v>915</v>
       </c>
       <c r="N213" s="19">
-        <v>193</v>
+        <v>245</v>
       </c>
     </row>
     <row r="214" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -14350,7 +14350,7 @@
         <v>915</v>
       </c>
       <c r="N214" s="19">
-        <v>114</v>
+        <v>131</v>
       </c>
     </row>
     <row r="215" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -14394,7 +14394,7 @@
         <v>915</v>
       </c>
       <c r="N215" s="19">
-        <v>264</v>
+        <v>184</v>
       </c>
     </row>
     <row r="216" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -14438,7 +14438,7 @@
         <v>915</v>
       </c>
       <c r="N216" s="19">
-        <v>82</v>
+        <v>179</v>
       </c>
     </row>
     <row r="217" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -14482,7 +14482,7 @@
         <v>915</v>
       </c>
       <c r="N217" s="19">
-        <v>158</v>
+        <v>134</v>
       </c>
     </row>
     <row r="218" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -14526,7 +14526,7 @@
         <v>915</v>
       </c>
       <c r="N218" s="19">
-        <v>281</v>
+        <v>245</v>
       </c>
     </row>
     <row r="219" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -14570,7 +14570,7 @@
         <v>915</v>
       </c>
       <c r="N219" s="19">
-        <v>97</v>
+        <v>131</v>
       </c>
     </row>
     <row r="220" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -14658,7 +14658,7 @@
         <v>915</v>
       </c>
       <c r="N221" s="19">
-        <v>109</v>
+        <v>279</v>
       </c>
     </row>
     <row r="222" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -14702,7 +14702,7 @@
         <v>915</v>
       </c>
       <c r="N222" s="19">
-        <v>199</v>
+        <v>230</v>
       </c>
     </row>
     <row r="223" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -14746,7 +14746,7 @@
         <v>915</v>
       </c>
       <c r="N223" s="19">
-        <v>302</v>
+        <v>195</v>
       </c>
     </row>
     <row r="224" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -14790,7 +14790,7 @@
         <v>915</v>
       </c>
       <c r="N224" s="19">
-        <v>230</v>
+        <v>267</v>
       </c>
     </row>
     <row r="225" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -14834,7 +14834,7 @@
         <v>915</v>
       </c>
       <c r="N225" s="19">
-        <v>304</v>
+        <v>213</v>
       </c>
     </row>
     <row r="226" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -14878,7 +14878,7 @@
         <v>915</v>
       </c>
       <c r="N226" s="19">
-        <v>80</v>
+        <v>201</v>
       </c>
     </row>
     <row r="227" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -14922,7 +14922,7 @@
         <v>915</v>
       </c>
       <c r="N227" s="19">
-        <v>173</v>
+        <v>257</v>
       </c>
     </row>
     <row r="228" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -14966,7 +14966,7 @@
         <v>915</v>
       </c>
       <c r="N228" s="19">
-        <v>288</v>
+        <v>242</v>
       </c>
     </row>
     <row r="229" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -15010,7 +15010,7 @@
         <v>915</v>
       </c>
       <c r="N229" s="19">
-        <v>263</v>
+        <v>280</v>
       </c>
     </row>
     <row r="230" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -15054,7 +15054,7 @@
         <v>915</v>
       </c>
       <c r="N230" s="19">
-        <v>206</v>
+        <v>121</v>
       </c>
     </row>
     <row r="231" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -15098,7 +15098,7 @@
         <v>915</v>
       </c>
       <c r="N231" s="19">
-        <v>132</v>
+        <v>174</v>
       </c>
     </row>
     <row r="232" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -15142,7 +15142,7 @@
         <v>1017</v>
       </c>
       <c r="N232" s="19">
-        <v>180</v>
+        <v>227</v>
       </c>
     </row>
     <row r="233" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -15186,7 +15186,7 @@
         <v>1017</v>
       </c>
       <c r="N233" s="19">
-        <v>243</v>
+        <v>269</v>
       </c>
     </row>
     <row r="234" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -15230,7 +15230,7 @@
         <v>1017</v>
       </c>
       <c r="N234" s="19">
-        <v>129</v>
+        <v>297</v>
       </c>
     </row>
     <row r="235" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -15274,7 +15274,7 @@
         <v>1017</v>
       </c>
       <c r="N235" s="19">
-        <v>250</v>
+        <v>180</v>
       </c>
     </row>
     <row r="236" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -15318,7 +15318,7 @@
         <v>1017</v>
       </c>
       <c r="N236" s="19">
-        <v>280</v>
+        <v>210</v>
       </c>
     </row>
     <row r="237" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -15362,7 +15362,7 @@
         <v>1017</v>
       </c>
       <c r="N237" s="19">
-        <v>192</v>
+        <v>241</v>
       </c>
     </row>
     <row r="238" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -15406,7 +15406,7 @@
         <v>1017</v>
       </c>
       <c r="N238" s="19">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="239" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -15450,7 +15450,7 @@
         <v>1017</v>
       </c>
       <c r="N239" s="19">
-        <v>298</v>
+        <v>81</v>
       </c>
     </row>
     <row r="240" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -15494,7 +15494,7 @@
         <v>1017</v>
       </c>
       <c r="N240" s="19">
-        <v>194</v>
+        <v>306</v>
       </c>
     </row>
     <row r="241" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -15538,7 +15538,7 @@
         <v>1017</v>
       </c>
       <c r="N241" s="19">
-        <v>160</v>
+        <v>172</v>
       </c>
     </row>
     <row r="242" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -15582,7 +15582,7 @@
         <v>1017</v>
       </c>
       <c r="N242" s="19">
-        <v>99</v>
+        <v>129</v>
       </c>
     </row>
     <row r="243" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -15626,7 +15626,7 @@
         <v>1017</v>
       </c>
       <c r="N243" s="19">
-        <v>221</v>
+        <v>90</v>
       </c>
     </row>
     <row r="244" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -15670,7 +15670,7 @@
         <v>1017</v>
       </c>
       <c r="N244" s="19">
-        <v>273</v>
+        <v>213</v>
       </c>
     </row>
     <row r="245" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -15714,7 +15714,7 @@
         <v>1017</v>
       </c>
       <c r="N245" s="19">
-        <v>60</v>
+        <v>253</v>
       </c>
     </row>
     <row r="246" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -15758,7 +15758,7 @@
         <v>1017</v>
       </c>
       <c r="N246" s="19">
-        <v>181</v>
+        <v>199</v>
       </c>
     </row>
     <row r="247" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -15802,7 +15802,7 @@
         <v>1017</v>
       </c>
       <c r="N247" s="19">
-        <v>66</v>
+        <v>125</v>
       </c>
     </row>
     <row r="248" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -15846,7 +15846,7 @@
         <v>1017</v>
       </c>
       <c r="N248" s="19">
-        <v>266</v>
+        <v>150</v>
       </c>
     </row>
     <row r="249" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -15890,7 +15890,7 @@
         <v>1017</v>
       </c>
       <c r="N249" s="19">
-        <v>266</v>
+        <v>162</v>
       </c>
     </row>
     <row r="250" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -15934,7 +15934,7 @@
         <v>1017</v>
       </c>
       <c r="N250" s="19">
-        <v>146</v>
+        <v>173</v>
       </c>
     </row>
     <row r="251" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -15978,7 +15978,7 @@
         <v>1017</v>
       </c>
       <c r="N251" s="19">
-        <v>230</v>
+        <v>303</v>
       </c>
     </row>
     <row r="252" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -16022,7 +16022,7 @@
         <v>1017</v>
       </c>
       <c r="N252" s="19">
-        <v>219</v>
+        <v>266</v>
       </c>
     </row>
     <row r="253" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -16066,7 +16066,7 @@
         <v>1017</v>
       </c>
       <c r="N253" s="19">
-        <v>113</v>
+        <v>174</v>
       </c>
     </row>
     <row r="254" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -16110,7 +16110,7 @@
         <v>1017</v>
       </c>
       <c r="N254" s="19">
-        <v>63</v>
+        <v>177</v>
       </c>
     </row>
     <row r="255" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -16154,7 +16154,7 @@
         <v>1017</v>
       </c>
       <c r="N255" s="19">
-        <v>116</v>
+        <v>79</v>
       </c>
     </row>
     <row r="256" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -16198,7 +16198,7 @@
         <v>1017</v>
       </c>
       <c r="N256" s="19">
-        <v>147</v>
+        <v>99</v>
       </c>
     </row>
     <row r="257" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -16242,7 +16242,7 @@
         <v>1017</v>
       </c>
       <c r="N257" s="19">
-        <v>69</v>
+        <v>244</v>
       </c>
     </row>
     <row r="258" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -16286,7 +16286,7 @@
         <v>1017</v>
       </c>
       <c r="N258" s="19">
-        <v>88</v>
+        <v>286</v>
       </c>
     </row>
     <row r="259" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -16330,7 +16330,7 @@
         <v>1017</v>
       </c>
       <c r="N259" s="19">
-        <v>153</v>
+        <v>214</v>
       </c>
     </row>
     <row r="260" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -16374,7 +16374,7 @@
         <v>1017</v>
       </c>
       <c r="N260" s="19">
-        <v>63</v>
+        <v>135</v>
       </c>
     </row>
     <row r="261" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -16418,7 +16418,7 @@
         <v>1017</v>
       </c>
       <c r="N261" s="19">
-        <v>145</v>
+        <v>302</v>
       </c>
     </row>
     <row r="262" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -16462,7 +16462,7 @@
         <v>1017</v>
       </c>
       <c r="N262" s="19">
-        <v>253</v>
+        <v>243</v>
       </c>
     </row>
     <row r="263" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -16506,7 +16506,7 @@
         <v>1017</v>
       </c>
       <c r="N263" s="19">
-        <v>71</v>
+        <v>251</v>
       </c>
     </row>
     <row r="264" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -16550,7 +16550,7 @@
         <v>1017</v>
       </c>
       <c r="N264" s="19">
-        <v>256</v>
+        <v>118</v>
       </c>
     </row>
     <row r="265" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -16594,7 +16594,7 @@
         <v>1017</v>
       </c>
       <c r="N265" s="19">
-        <v>245</v>
+        <v>122</v>
       </c>
     </row>
     <row r="266" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -16638,7 +16638,7 @@
         <v>1017</v>
       </c>
       <c r="N266" s="19">
-        <v>139</v>
+        <v>86</v>
       </c>
     </row>
     <row r="267" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -16682,7 +16682,7 @@
         <v>1159</v>
       </c>
       <c r="N267" s="19">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="268" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -16726,7 +16726,7 @@
         <v>1159</v>
       </c>
       <c r="N268" s="19">
-        <v>181</v>
+        <v>164</v>
       </c>
     </row>
     <row r="269" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -16770,7 +16770,7 @@
         <v>1159</v>
       </c>
       <c r="N269" s="19">
-        <v>142</v>
+        <v>162</v>
       </c>
     </row>
     <row r="270" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -16814,7 +16814,7 @@
         <v>1159</v>
       </c>
       <c r="N270" s="19">
-        <v>106</v>
+        <v>246</v>
       </c>
     </row>
     <row r="271" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -16858,7 +16858,7 @@
         <v>1159</v>
       </c>
       <c r="N271" s="19">
-        <v>105</v>
+        <v>164</v>
       </c>
     </row>
     <row r="272" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -16902,7 +16902,7 @@
         <v>1159</v>
       </c>
       <c r="N272" s="19">
-        <v>300</v>
+        <v>161</v>
       </c>
     </row>
     <row r="273" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -16946,7 +16946,7 @@
         <v>1159</v>
       </c>
       <c r="N273" s="19">
-        <v>85</v>
+        <v>203</v>
       </c>
     </row>
     <row r="274" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -16990,7 +16990,7 @@
         <v>1159</v>
       </c>
       <c r="N274" s="19">
-        <v>272</v>
+        <v>207</v>
       </c>
     </row>
     <row r="275" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -17034,7 +17034,7 @@
         <v>1159</v>
       </c>
       <c r="N275" s="19">
-        <v>153</v>
+        <v>122</v>
       </c>
     </row>
     <row r="276" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -17078,7 +17078,7 @@
         <v>1159</v>
       </c>
       <c r="N276" s="19">
-        <v>302</v>
+        <v>258</v>
       </c>
     </row>
     <row r="277" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -17122,7 +17122,7 @@
         <v>1159</v>
       </c>
       <c r="N277" s="19">
-        <v>242</v>
+        <v>176</v>
       </c>
     </row>
     <row r="278" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -17166,7 +17166,7 @@
         <v>1159</v>
       </c>
       <c r="N278" s="19">
-        <v>106</v>
+        <v>85</v>
       </c>
     </row>
     <row r="279" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -17210,7 +17210,7 @@
         <v>1159</v>
       </c>
       <c r="N279" s="19">
-        <v>93</v>
+        <v>268</v>
       </c>
     </row>
     <row r="280" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -17254,7 +17254,7 @@
         <v>1159</v>
       </c>
       <c r="N280" s="19">
-        <v>216</v>
+        <v>172</v>
       </c>
     </row>
     <row r="281" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -17298,7 +17298,7 @@
         <v>1159</v>
       </c>
       <c r="N281" s="19">
-        <v>287</v>
+        <v>90</v>
       </c>
     </row>
     <row r="282" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -17342,7 +17342,7 @@
         <v>1159</v>
       </c>
       <c r="N282" s="19">
-        <v>76</v>
+        <v>89</v>
       </c>
     </row>
     <row r="283" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -17386,7 +17386,7 @@
         <v>1159</v>
       </c>
       <c r="N283" s="19">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="284" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -17430,7 +17430,7 @@
         <v>1159</v>
       </c>
       <c r="N284" s="19">
-        <v>73</v>
+        <v>150</v>
       </c>
     </row>
     <row r="285" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -17474,7 +17474,7 @@
         <v>1159</v>
       </c>
       <c r="N285" s="19">
-        <v>189</v>
+        <v>143</v>
       </c>
     </row>
     <row r="286" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -17518,7 +17518,7 @@
         <v>1159</v>
       </c>
       <c r="N286" s="19">
-        <v>125</v>
+        <v>152</v>
       </c>
     </row>
     <row r="287" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -17562,7 +17562,7 @@
         <v>1159</v>
       </c>
       <c r="N287" s="19">
-        <v>141</v>
+        <v>246</v>
       </c>
     </row>
     <row r="288" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -17606,7 +17606,7 @@
         <v>1159</v>
       </c>
       <c r="N288" s="19">
-        <v>193</v>
+        <v>75</v>
       </c>
     </row>
     <row r="289" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -17650,7 +17650,7 @@
         <v>1159</v>
       </c>
       <c r="N289" s="19">
-        <v>287</v>
+        <v>92</v>
       </c>
     </row>
     <row r="290" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -17694,7 +17694,7 @@
         <v>1159</v>
       </c>
       <c r="N290" s="19">
-        <v>94</v>
+        <v>181</v>
       </c>
     </row>
     <row r="291" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -17738,7 +17738,7 @@
         <v>1159</v>
       </c>
       <c r="N291" s="19">
-        <v>228</v>
+        <v>178</v>
       </c>
     </row>
     <row r="292" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -17782,7 +17782,7 @@
         <v>1159</v>
       </c>
       <c r="N292" s="19">
-        <v>240</v>
+        <v>123</v>
       </c>
     </row>
     <row r="293" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -17826,7 +17826,7 @@
         <v>1159</v>
       </c>
       <c r="N293" s="19">
-        <v>297</v>
+        <v>122</v>
       </c>
     </row>
     <row r="294" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -17870,7 +17870,7 @@
         <v>1159</v>
       </c>
       <c r="N294" s="19">
-        <v>88</v>
+        <v>72</v>
       </c>
     </row>
     <row r="295" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -17958,7 +17958,7 @@
         <v>1159</v>
       </c>
       <c r="N296" s="19">
-        <v>267</v>
+        <v>108</v>
       </c>
     </row>
     <row r="297" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -18002,7 +18002,7 @@
         <v>1159</v>
       </c>
       <c r="N297" s="19">
-        <v>187</v>
+        <v>68</v>
       </c>
     </row>
     <row r="298" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -18046,7 +18046,7 @@
         <v>1159</v>
       </c>
       <c r="N298" s="19">
-        <v>246</v>
+        <v>181</v>
       </c>
     </row>
     <row r="299" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -18090,7 +18090,7 @@
         <v>1159</v>
       </c>
       <c r="N299" s="19">
-        <v>123</v>
+        <v>304</v>
       </c>
     </row>
     <row r="300" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -18134,7 +18134,7 @@
         <v>1159</v>
       </c>
       <c r="N300" s="19">
-        <v>186</v>
+        <v>67</v>
       </c>
     </row>
     <row r="301" spans="1:14" s="19" customFormat="1" x14ac:dyDescent="0.25">
@@ -18178,7 +18178,7 @@
         <v>1159</v>
       </c>
       <c r="N301" s="19">
-        <v>269</v>
+        <v>189</v>
       </c>
     </row>
   </sheetData>

</xml_diff>